<commit_message>
Doc: where the problem sits in Operations Management (checked against our numbers); matrix counts from the dataset; tray weights; refreshed results
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013JwSYm4UV7vKHqaUukbU1G
</commit_message>
<xml_diff>
--- a/docs/MDS_Decision_Workbook.xlsx
+++ b/docs/MDS_Decision_Workbook.xlsx
@@ -102,7 +102,7 @@
     <t xml:space="preserve">Output of our prototype's simulator</t>
   </si>
   <si>
-    <t xml:space="preserve">Average wait 7.2 → 0.8 min</t>
+    <t xml:space="preserve">Average wait 7.2 → 1.1 min</t>
   </si>
   <si>
     <t xml:space="preserve">Tabs and course sessions</t>
@@ -1278,7 +1278,7 @@
     <t xml:space="preserve">Session 7: Decision making under certainty, risk and uncertainty (maximax, maximin, minimax regret, Hurwicz, Laplace, EMV, EVPI)</t>
   </si>
   <si>
-    <t xml:space="preserve">Everything on this tab is in MINUTES of waiting per student, so no rupee values are needed. Blue = input. S2 values for A1 and A2 come from our simulator (7.2 → 0.8 min); the other cells are illustrative estimates.</t>
+    <t xml:space="preserve">Everything on this tab is in MINUTES of waiting per student, so no rupee values are needed. Blue = input. S2 values for A1 and A2 come from our simulator (7.2 → 1.1 min); the other cells are illustrative estimates.</t>
   </si>
   <si>
     <t xml:space="preserve">Average wait per student (minutes)  [lower is better]</t>
@@ -1782,7 +1782,7 @@
     <t xml:space="preserve">Best alternative (AHP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Service-level scores can be anchored to the queuing results (S15) and the payoff matrix (S7): e.g. average wait 7.2 min → 3, 0.8 min → 8. Criteria come from our Phase 1 deck's weighted decision table.</t>
+    <t xml:space="preserve">Service-level scores can be anchored to the queuing results (S15) and the payoff matrix (S7): e.g. average wait 7.2 min → 3, 1.1 min → 8. Criteria come from our Phase 1 deck's weighted decision table.</t>
   </si>
   <si>
     <t xml:space="preserve">Best–Worst Method: the same criteria weights with fewer comparisons</t>
@@ -2088,7 +2088,7 @@
     <t xml:space="preserve">The spreadsheet model is simpler than the simulator (fixed 10-min bins, no stock-outs, no seat limit), so the two will not match exactly; both should show the same direction and rough size of improvement.</t>
   </si>
   <si>
-    <t xml:space="preserve">Findings from the simulator: (1) Moving students moves the food run-outs: with screens Munch feeds more students and a 30-min call-back restock cannot keep up, so routing and food allocation (S10-11 LP) must be planned together; if the next batch is always made before the call (10–14 min to send), run-outs disappear in the model (table below). (2) The single face scanner (~30 scans/min at an assumed 2 s each) is close to Central's peak arrival rate, so a queue of 20–25 people can form OUTSIDE the scanner, which the biometric data cannot see.</t>
+    <t xml:space="preserve">Findings from the simulator: (1) Routing and food interact: when the next batch is rarely ready, run-outs stay about the same with screens (Munch feeds more students and a 30-min call-back cannot keep up); when food is usually ready, screens cut run-outs, because a star dish marked 'out' sends students to the other mess at once. Plan routing and food allocation (S10-11 LP) together; if the next batch is always made before the call (10–14 min), run-outs disappear (table below). (2) The single face scanner (~30 scans/min at an assumed 2 s each) is close to Central's peak arrival rate, so a queue of 20–25 people can form OUTSIDE the scanner, which the biometric data cannot see.</t>
   </si>
   <si>
     <t xml:space="preserve">Next batch already made when the mess calls?</t>
@@ -2878,11 +2878,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="62409454"/>
-        <c:axId val="29120686"/>
+        <c:axId val="21186051"/>
+        <c:axId val="36980189"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="62409454"/>
+        <c:axId val="21186051"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2948,7 +2948,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29120686"/>
+        <c:crossAx val="36980189"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2956,7 +2956,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="29120686"/>
+        <c:axId val="36980189"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3032,7 +3032,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62409454"/>
+        <c:crossAx val="21186051"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3832,11 +3832,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="48426104"/>
-        <c:axId val="91551624"/>
+        <c:axId val="78154611"/>
+        <c:axId val="73859903"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="48426104"/>
+        <c:axId val="78154611"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3868,7 +3868,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91551624"/>
+        <c:crossAx val="73859903"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3876,7 +3876,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="91551624"/>
+        <c:axId val="73859903"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3952,7 +3952,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48426104"/>
+        <c:crossAx val="78154611"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4130,16 +4130,16 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.54</c:v>
+                  <c:v>5.33</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6.04</c:v>
+                  <c:v>5.83</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>3.35</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6</c:v>
+                  <c:v>5.87</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4147,11 +4147,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="74992750"/>
-        <c:axId val="66402931"/>
+        <c:axId val="25705602"/>
+        <c:axId val="23205098"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="74992750"/>
+        <c:axId val="25705602"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4183,7 +4183,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66402931"/>
+        <c:crossAx val="23205098"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4191,7 +4191,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="66402931"/>
+        <c:axId val="23205098"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4233,7 +4233,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74992750"/>
+        <c:crossAx val="25705602"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4589,11 +4589,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="61766926"/>
-        <c:axId val="59186027"/>
+        <c:axId val="53313538"/>
+        <c:axId val="95202996"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="61766926"/>
+        <c:axId val="53313538"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4625,7 +4625,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59186027"/>
+        <c:crossAx val="95202996"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4633,7 +4633,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="59186027"/>
+        <c:axId val="95202996"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4675,7 +4675,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61766926"/>
+        <c:crossAx val="53313538"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4907,11 +4907,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="19812427"/>
-        <c:axId val="70670018"/>
+        <c:axId val="65048712"/>
+        <c:axId val="84066847"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="19812427"/>
+        <c:axId val="65048712"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4987,12 +4987,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="70670018"/>
+        <c:crossAx val="84066847"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="70670018"/>
+        <c:axId val="84066847"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5068,7 +5068,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19812427"/>
+        <c:crossAx val="65048712"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5219,13 +5219,13 @@
                   <c:v>7.2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.4</c:v>
+                  <c:v>1.6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.8</c:v>
+                  <c:v>1.1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.9</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5233,11 +5233,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="22127919"/>
-        <c:axId val="95985930"/>
+        <c:axId val="97367826"/>
+        <c:axId val="94085906"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="22127919"/>
+        <c:axId val="97367826"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5269,7 +5269,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95985930"/>
+        <c:crossAx val="94085906"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5277,7 +5277,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="95985930"/>
+        <c:axId val="94085906"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5319,7 +5319,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22127919"/>
+        <c:crossAx val="97367826"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -10338,10 +10338,10 @@
         <v>658</v>
       </c>
       <c r="B22" s="37" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="C22" s="37" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="D22" s="8" t="s">
         <v>659</v>
@@ -10352,10 +10352,10 @@
         <v>660</v>
       </c>
       <c r="B23" s="37" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="C23" s="37" t="n">
-        <v>2.5</v>
+        <v>3.1</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>661</v>
@@ -10472,19 +10472,19 @@
         <v>0.3</v>
       </c>
       <c r="C6" s="37" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="D6" s="37" t="n">
-        <v>4.3</v>
+        <v>4.8</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="G6" s="37" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10495,19 +10495,19 @@
         <v>0.6</v>
       </c>
       <c r="C7" s="37" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="D7" s="37" t="n">
-        <v>2.5</v>
+        <v>3.1</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="G7" s="37" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10518,19 +10518,19 @@
         <v>1</v>
       </c>
       <c r="C8" s="37" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="D8" s="37" t="n">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G8" s="37" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10539,7 +10539,7 @@
       </c>
       <c r="C10" s="62" t="n">
         <f aca="false">1-C7/C5</f>
-        <v>0.888888888888889</v>
+        <v>0.847222222222222</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10647,13 +10647,13 @@
         <v>2</v>
       </c>
       <c r="D25" s="37" t="n">
-        <v>3</v>
+        <v>2.1</v>
       </c>
       <c r="E25" s="37" t="n">
         <v>7</v>
       </c>
       <c r="F25" s="37" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10667,13 +10667,13 @@
         <v>1.3</v>
       </c>
       <c r="D26" s="37" t="n">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
       <c r="E26" s="37" t="n">
         <v>7.1</v>
       </c>
       <c r="F26" s="37" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10687,13 +10687,13 @@
         <v>0.8</v>
       </c>
       <c r="D27" s="37" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="E27" s="37" t="n">
         <v>7.2</v>
       </c>
       <c r="F27" s="37" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15741,10 +15741,10 @@
         <v>306</v>
       </c>
       <c r="B8" s="37" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="C8" s="37" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="D8" s="37" t="n">
         <v>6</v>
@@ -15760,10 +15760,10 @@
         <v>309</v>
       </c>
       <c r="B9" s="37" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="C9" s="37" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="D9" s="37" t="n">
         <v>3.5</v>
@@ -15798,10 +15798,10 @@
         <v>422</v>
       </c>
       <c r="B11" s="37" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="C11" s="37" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="D11" s="37" t="n">
         <v>4.5</v>
@@ -15935,11 +15935,11 @@
       </c>
       <c r="B20" s="22" t="n">
         <f aca="false">B$7-B8</f>
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="C20" s="22" t="n">
         <f aca="false">C$7-C8</f>
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="D20" s="22" t="n">
         <f aca="false">D$7-D8</f>
@@ -15951,23 +15951,23 @@
       </c>
       <c r="F20" s="22" t="n">
         <f aca="false">MIN(B20:D20)</f>
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="G20" s="22" t="n">
         <f aca="false">$B$26*E20+(1-$B$26)*F20</f>
-        <v>4.68</v>
+        <v>4.56</v>
       </c>
       <c r="H20" s="22" t="n">
         <f aca="false">AVERAGE(B20:D20)</f>
-        <v>5.73333333333333</v>
+        <v>5.56666666666667</v>
       </c>
       <c r="I20" s="29" t="n">
         <f aca="false">SUMPRODUCT(B20:D20,$B$14:$D$14)</f>
-        <v>5.54</v>
+        <v>5.33</v>
       </c>
       <c r="J20" s="40" t="n">
         <f aca="false">I20*$B$15/60</f>
-        <v>273.306666666667</v>
+        <v>262.946666666667</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15976,11 +15976,11 @@
       </c>
       <c r="B21" s="22" t="n">
         <f aca="false">B$7-B9</f>
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="C21" s="22" t="n">
         <f aca="false">C$7-C9</f>
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="D21" s="22" t="n">
         <f aca="false">D$7-D9</f>
@@ -15992,23 +15992,23 @@
       </c>
       <c r="F21" s="22" t="n">
         <f aca="false">MIN(B21:D21)</f>
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="G21" s="22" t="n">
         <f aca="false">$B$26*E21+(1-$B$26)*F21</f>
-        <v>5.68</v>
+        <v>5.56</v>
       </c>
       <c r="H21" s="22" t="n">
         <f aca="false">AVERAGE(B21:D21)</f>
-        <v>6.56666666666667</v>
+        <v>6.4</v>
       </c>
       <c r="I21" s="29" t="n">
         <f aca="false">SUMPRODUCT(B21:D21,$B$14:$D$14)</f>
-        <v>6.04</v>
+        <v>5.83</v>
       </c>
       <c r="J21" s="40" t="n">
         <f aca="false">I21*$B$15/60</f>
-        <v>297.973333333333</v>
+        <v>287.613333333333</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16058,11 +16058,11 @@
       </c>
       <c r="B23" s="22" t="n">
         <f aca="false">B$7-B11</f>
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="C23" s="22" t="n">
         <f aca="false">C$7-C11</f>
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="D23" s="22" t="n">
         <f aca="false">D$7-D11</f>
@@ -16074,23 +16074,23 @@
       </c>
       <c r="F23" s="22" t="n">
         <f aca="false">MIN(B23:D23)</f>
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="G23" s="22" t="n">
         <f aca="false">$B$26*E23+(1-$B$26)*F23</f>
-        <v>5.4</v>
+        <v>5.34</v>
       </c>
       <c r="H23" s="22" t="n">
         <f aca="false">AVERAGE(B23:D23)</f>
-        <v>6.36666666666667</v>
+        <v>6.26666666666667</v>
       </c>
       <c r="I23" s="29" t="n">
         <f aca="false">SUMPRODUCT(B23:D23,$B$14:$D$14)</f>
-        <v>6</v>
+        <v>5.87</v>
       </c>
       <c r="J23" s="40" t="n">
         <f aca="false">I23*$B$15/60</f>
-        <v>296</v>
+        <v>289.586666666667</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16115,7 +16115,7 @@
       </c>
       <c r="I24" s="41" t="str">
         <f aca="false">INDEX($A$19:$A$23,MATCH(MAX(I19:I23),I19:I23,0))</f>
-        <v>A3 Screens + kitchen early alerts</v>
+        <v>A5 Screens + 3rd serving station</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16157,11 +16157,11 @@
       </c>
       <c r="B30" s="22" t="n">
         <f aca="false">MAX(B$19:B$23)-B19</f>
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="C30" s="22" t="n">
         <f aca="false">MAX(C$19:C$23)-C19</f>
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="D30" s="22" t="n">
         <f aca="false">MAX(D$19:D$23)-D19</f>
@@ -16173,7 +16173,7 @@
       </c>
       <c r="F30" s="29" t="n">
         <f aca="false">SUMPRODUCT(B30:D30,$B$14:$D$14)</f>
-        <v>6.2</v>
+        <v>6.07</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16182,11 +16182,11 @@
       </c>
       <c r="B31" s="22" t="n">
         <f aca="false">MAX(B$19:B$23)-B20</f>
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="C31" s="22" t="n">
         <f aca="false">MAX(C$19:C$23)-C20</f>
-        <v>0.2</v>
+        <v>0.300000000000001</v>
       </c>
       <c r="D31" s="22" t="n">
         <f aca="false">MAX(D$19:D$23)-D20</f>
@@ -16198,7 +16198,7 @@
       </c>
       <c r="F31" s="29" t="n">
         <f aca="false">SUMPRODUCT(B31:D31,$B$14:$D$14)</f>
-        <v>0.66</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16207,11 +16207,11 @@
       </c>
       <c r="B32" s="22" t="n">
         <f aca="false">MAX(B$19:B$23)-B21</f>
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="C32" s="22" t="n">
         <f aca="false">MAX(C$19:C$23)-C21</f>
-        <v>0.2</v>
+        <v>0.300000000000001</v>
       </c>
       <c r="D32" s="22" t="n">
         <f aca="false">MAX(D$19:D$23)-D21</f>
@@ -16219,11 +16219,11 @@
       </c>
       <c r="E32" s="22" t="n">
         <f aca="false">MAX(B32:D32)</f>
-        <v>0.2</v>
+        <v>0.300000000000001</v>
       </c>
       <c r="F32" s="29" t="n">
         <f aca="false">SUMPRODUCT(B32:D32,$B$14:$D$14)</f>
-        <v>0.16</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16232,11 +16232,11 @@
       </c>
       <c r="B33" s="22" t="n">
         <f aca="false">MAX(B$19:B$23)-B22</f>
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="C33" s="22" t="n">
         <f aca="false">MAX(C$19:C$23)-C22</f>
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
       <c r="D33" s="22" t="n">
         <f aca="false">MAX(D$19:D$23)-D22</f>
@@ -16248,7 +16248,7 @@
       </c>
       <c r="F33" s="29" t="n">
         <f aca="false">SUMPRODUCT(B33:D33,$B$14:$D$14)</f>
-        <v>2.85</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16291,7 +16291,7 @@
       </c>
       <c r="F36" s="41" t="str">
         <f aca="false">INDEX($A$30:$A$34,MATCH(MIN(F30:F34),F30:F34,0))</f>
-        <v>A3 Screens + kitchen early alerts</v>
+        <v>A5 Screens + 3rd serving station</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16305,7 +16305,7 @@
       </c>
       <c r="B39" s="29" t="n">
         <f aca="false">B14*MAX(B19:B23)+C14*MAX(C19:C23)+D14*MAX(D19:D23)</f>
-        <v>6.2</v>
+        <v>6.07</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16314,7 +16314,7 @@
       </c>
       <c r="B40" s="29" t="n">
         <f aca="false">MAX(I19:I23)</f>
-        <v>6.04</v>
+        <v>5.87</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16323,7 +16323,7 @@
       </c>
       <c r="B41" s="42" t="n">
         <f aca="false">B39-B40</f>
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16332,7 +16332,7 @@
       </c>
       <c r="B42" s="29" t="n">
         <f aca="false">MIN(F30:F34)</f>
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
New project title (Beyond the Bottleneck) and revised problem statement; Phase 1 to Phase 2 bridge
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013JwSYm4UV7vKHqaUukbU1G
</commit_message>
<xml_diff>
--- a/docs/MDS_Decision_Workbook.xlsx
+++ b/docs/MDS_Decision_Workbook.xlsx
@@ -36,10 +36,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="699">
   <si>
-    <t xml:space="preserve">MDS decision workbook — Mess queue and allocation project (Group WGB3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every Management Decision Science course topic applied to the Chefs Touch lunch problem (Central CT and Munch Mess, lunch 11:30–14:30).</t>
+    <t xml:space="preserve">MDS decision workbook — Beyond the Bottleneck (Group WGB3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beyond the Bottleneck: Enabling Smarter Lunch Flow by Optimising Queue Management and Capacity Utilisation Across Chefs Touch Centres. Every MDS course topic applied (Central CT and Munch Mess, lunch 11:30–14:30).</t>
   </si>
   <si>
     <t xml:space="preserve">How to use</t>
@@ -501,10 +501,10 @@
     <t xml:space="preserve">Sessions 2–3: Nature of business decisions · Problem identification, structuring, root cause analysis</t>
   </si>
   <si>
-    <t xml:space="preserve">Problem statement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">During the 11:30–14:30 lunch window, Chefs Touch serves about 2,960 plates. Demand is concentrated while kitchen, delivery and serving capacity are fixed, so students wait (~15 min observed), star dishes run out mid-service and replenishment arrives during the peak. Decision question: are resources (food, serving lines, students' choice of mess) reaching the right centre, in the right quantity, at the right time?</t>
+    <t xml:space="preserve">Problem statement (Phase 2: Beyond the Bottleneck)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">During the 11:30–14:30 lunch window, Chefs Touch serves about 2,960 students. Total serving capacity is enough on average but is used unevenly: one centre is saturated while another has spare capacity, so students wait (~15 min observed) and star-dish run-outs at the busy centre make it worse. Decision question: how should student flow and serving capacity be balanced across CT's centres, minute by minute, so that waiting falls without adding staff or space? (Phase 1, 'The Two-Hour Bottleneck', asked whether food reached the right centre in the right quantity at the right time; that question continues in S7 and S10-11.)</t>
   </si>
   <si>
     <t xml:space="preserve">Session 2: nature of the decision</t>
@@ -2878,11 +2878,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="21186051"/>
-        <c:axId val="36980189"/>
+        <c:axId val="41725249"/>
+        <c:axId val="33609352"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="21186051"/>
+        <c:axId val="41725249"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2948,7 +2948,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36980189"/>
+        <c:crossAx val="33609352"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2956,7 +2956,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="36980189"/>
+        <c:axId val="33609352"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3032,7 +3032,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21186051"/>
+        <c:crossAx val="41725249"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3832,11 +3832,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="78154611"/>
-        <c:axId val="73859903"/>
+        <c:axId val="42397101"/>
+        <c:axId val="96811856"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="78154611"/>
+        <c:axId val="42397101"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3868,7 +3868,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="73859903"/>
+        <c:crossAx val="96811856"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3876,7 +3876,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="73859903"/>
+        <c:axId val="96811856"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3952,7 +3952,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78154611"/>
+        <c:crossAx val="42397101"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4147,11 +4147,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="25705602"/>
-        <c:axId val="23205098"/>
+        <c:axId val="76788725"/>
+        <c:axId val="43018370"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="25705602"/>
+        <c:axId val="76788725"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4183,7 +4183,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23205098"/>
+        <c:crossAx val="43018370"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4191,7 +4191,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="23205098"/>
+        <c:axId val="43018370"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4233,7 +4233,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25705602"/>
+        <c:crossAx val="76788725"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4589,11 +4589,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="53313538"/>
-        <c:axId val="95202996"/>
+        <c:axId val="3830711"/>
+        <c:axId val="5675616"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="53313538"/>
+        <c:axId val="3830711"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4625,7 +4625,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95202996"/>
+        <c:crossAx val="5675616"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4633,7 +4633,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="95202996"/>
+        <c:axId val="5675616"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4675,7 +4675,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53313538"/>
+        <c:crossAx val="3830711"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4907,11 +4907,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="65048712"/>
-        <c:axId val="84066847"/>
+        <c:axId val="23516426"/>
+        <c:axId val="92118349"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="65048712"/>
+        <c:axId val="23516426"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4987,12 +4987,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84066847"/>
+        <c:crossAx val="92118349"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="84066847"/>
+        <c:axId val="92118349"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5068,7 +5068,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65048712"/>
+        <c:crossAx val="23516426"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5233,11 +5233,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="97367826"/>
-        <c:axId val="94085906"/>
+        <c:axId val="46110289"/>
+        <c:axId val="19228237"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="97367826"/>
+        <c:axId val="46110289"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5269,7 +5269,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94085906"/>
+        <c:crossAx val="19228237"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5277,7 +5277,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="94085906"/>
+        <c:axId val="19228237"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5319,7 +5319,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97367826"/>
+        <c:crossAx val="46110289"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5747,7 +5747,7 @@
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -11404,7 +11404,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
         <v>156</v>
       </c>

</xml_diff>

<commit_message>
Queue, capacity and load-balancing workbook on simulated data; Munch seats 492
New docs/Queue_Capacity_LoadBalancing.xlsx (tools/queue_capacity_data.py +
tools/build_queue_capacity_workbook.py): M/M/1 for the face scanner and
M/M/c for the serving stations per 10-min slot with stability and Little's
Law checks, seats as M/G/c and disposal as M/G/inf, seat turnover and the
bottleneck, and dynamic Smart Scan routing against static rules (freshers
at Munch, department assignments, fixed shares) across kinds of day.
The simulator records service end times and can run static department
assignments. Munch seats recounted to 492 (results unchanged: seats never
bind).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013JwSYm4UV7vKHqaUukbU1G
</commit_message>
<xml_diff>
--- a/docs/MDS_Decision_Workbook.xlsx
+++ b/docs/MDS_Decision_Workbook.xlsx
@@ -276,7 +276,7 @@
     <t xml:space="preserve">From field work, CT or the group</t>
   </si>
   <si>
-    <t xml:space="preserve">2,960 students; seats 900 / 500; 2 stations + 1 scanner per mess</t>
+    <t xml:space="preserve">2,960 students; seats 900 / 492; 2 stations + 1 scanner per mess</t>
   </si>
   <si>
     <t xml:space="preserve">Group estimate</t>
@@ -2985,7 +2985,7 @@
     <t xml:space="preserve">Stage 3: eating</t>
   </si>
   <si>
-    <t xml:space="preserve">Take a seat if free (900 / 500), else wait; eat for uniform 12–15 min</t>
+    <t xml:space="preserve">Take a seat if free (900 / 492), else wait; eat for uniform 12–15 min</t>
   </si>
   <si>
     <t xml:space="preserve">seats, eat_lo/hi</t>
@@ -5336,11 +5336,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="48609536"/>
-        <c:axId val="61275530"/>
+        <c:axId val="50982440"/>
+        <c:axId val="10555494"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="48609536"/>
+        <c:axId val="50982440"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5372,7 +5372,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61275530"/>
+        <c:crossAx val="10555494"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5380,7 +5380,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="61275530"/>
+        <c:axId val="10555494"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5456,7 +5456,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48609536"/>
+        <c:crossAx val="50982440"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5704,11 +5704,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="45861843"/>
-        <c:axId val="62849978"/>
+        <c:axId val="83326717"/>
+        <c:axId val="40401674"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="45861843"/>
+        <c:axId val="83326717"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5774,7 +5774,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62849978"/>
+        <c:crossAx val="40401674"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5782,7 +5782,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="62849978"/>
+        <c:axId val="40401674"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5858,7 +5858,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="45861843"/>
+        <c:crossAx val="83326717"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6658,11 +6658,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="12605798"/>
-        <c:axId val="55105881"/>
+        <c:axId val="35481415"/>
+        <c:axId val="88590308"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="12605798"/>
+        <c:axId val="35481415"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6694,7 +6694,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55105881"/>
+        <c:crossAx val="88590308"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6702,7 +6702,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="55105881"/>
+        <c:axId val="88590308"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6778,7 +6778,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12605798"/>
+        <c:crossAx val="35481415"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7422,11 +7422,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="36984693"/>
-        <c:axId val="90611264"/>
+        <c:axId val="47636435"/>
+        <c:axId val="43479"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="36984693"/>
+        <c:axId val="47636435"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7458,7 +7458,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90611264"/>
+        <c:crossAx val="43479"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7466,7 +7466,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="90611264"/>
+        <c:axId val="43479"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7542,7 +7542,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36984693"/>
+        <c:crossAx val="47636435"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7737,11 +7737,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="88720546"/>
-        <c:axId val="41637514"/>
+        <c:axId val="28356669"/>
+        <c:axId val="68303611"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="88720546"/>
+        <c:axId val="28356669"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7773,7 +7773,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41637514"/>
+        <c:crossAx val="68303611"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7781,7 +7781,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="41637514"/>
+        <c:axId val="68303611"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7823,7 +7823,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88720546"/>
+        <c:crossAx val="28356669"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7988,11 +7988,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="64340041"/>
-        <c:axId val="33257741"/>
+        <c:axId val="26361118"/>
+        <c:axId val="73593723"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="64340041"/>
+        <c:axId val="26361118"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8024,7 +8024,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33257741"/>
+        <c:crossAx val="73593723"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8032,7 +8032,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="33257741"/>
+        <c:axId val="73593723"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8074,7 +8074,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64340041"/>
+        <c:crossAx val="26361118"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -13115,7 +13115,7 @@
       <c r="F39" s="5"/>
       <c r="G39" s="31" t="n">
         <f aca="false">Inputs!$B$9/(Inputs!$B$9+Inputs!$B$10)</f>
-        <v>0.642857142857143</v>
+        <v>0.646551724137931</v>
       </c>
       <c r="H39" s="31"/>
       <c r="I39" s="31"/>
@@ -13805,7 +13805,7 @@
         <v>105</v>
       </c>
       <c r="B10" s="14" t="n">
-        <v>500</v>
+        <v>492</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>102</v>
@@ -15455,7 +15455,7 @@
       </c>
       <c r="B92" s="27" t="n">
         <f aca="false">Inputs!$B$10/Inputs!$B$87</f>
-        <v>37.037037037037</v>
+        <v>36.4444444444444</v>
       </c>
       <c r="C92" s="13" t="s">
         <v>138</v>
@@ -21628,7 +21628,7 @@
       </c>
       <c r="F58" s="32" t="n">
         <f aca="false">Inputs!$B$10</f>
-        <v>500</v>
+        <v>492</v>
       </c>
       <c r="G58" s="32" t="n">
         <f aca="false">Inputs!$B$9</f>
@@ -21636,7 +21636,7 @@
       </c>
       <c r="H58" s="32" t="n">
         <f aca="false">Inputs!$B$10</f>
-        <v>500</v>
+        <v>492</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>